<commit_message>
produktjakt 2026-09-11: slutbatch 15 (7 exploit / 5 explore / 3 säsong, 5 skyddsformer = 33 %) efter linser E+F — sida v16
- lins E (ordning/flerköp, maskinen gör jobbet): vedställsbeslag, kajakhållare, snöskyffel Makita, kedjeslipmaskin (K0-struken)
- lins F (synlig nyhet, kroppsligt, fars dag): garageportsnöflingor, värmesits älgpass, täljset, fågelmatare med kamera
- rank.py formtak lyfte batchen till 15 med 10 rader utan överdrag; dinosauriekalendern utanför (säsongstaket), registret uppdaterat
- STATUS-v3, LEARNING_STATE-raden, RUTIN-KVITTO uppdaterade

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MTP44ioo6XVSGukBjNdPXy
</commit_message>
<xml_diff>
--- a/produktjakt/korningar/2026-09-11/Leverantorsoffert-2026-09-11-v3.xlsx
+++ b/produktjakt/korningar/2026-09-11/Leverantorsoffert-2026-09-11-v3.xlsx
@@ -732,7 +732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU48"/>
+  <dimension ref="A1:AU64"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="18" customWidth="1" style="71" min="1" max="1"/>
@@ -767,7 +767,7 @@
   <sheetData>
     <row r="1" ht="27.75" customHeight="1" s="71">
       <c r="A1" s="1" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="AP1" s="1" t="n"/>
       <c r="AQ1" s="1" t="n"/>
@@ -1369,12 +1369,12 @@
       <c r="A13" s="10" t="n"/>
       <c r="D13" s="18" t="inlineStr">
         <is>
-          <t>Värmepumpsskyddet i aluminium</t>
+          <t>Snöflingor till garageporten 25-pack</t>
         </is>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $47.29. Vår räkning: landad ca 684 kr, tänkt butikspris 1499 kr. Originaltitel: Värmepumpsskyddet i aluminium</t>
+          <t>AliExpress: US $9.89. Vår räkning: landad ca 143 kr, tänkt butikspris 349 kr. Originaltitel: Snöflingor till garageporten 25-pack</t>
         </is>
       </c>
       <c r="H13" s="13" t="n"/>
@@ -1389,7 +1389,7 @@
       <c r="M13" s="14" t="n"/>
       <c r="N13" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012880367856.html</t>
+          <t>https://www.aliexpress.com/item/1005012790049322.html</t>
         </is>
       </c>
       <c r="Q13" s="18" t="n"/>
@@ -1539,12 +1539,12 @@
       <c r="A17" s="10" t="n"/>
       <c r="D17" s="18" t="inlineStr">
         <is>
-          <t>Takluckehuven 40×40, 2-pack</t>
+          <t>Värmepumpsskyddet i aluminium</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $4.75. Vår räkning: landad ca 138 kr, tänkt butikspris 499 kr. Originaltitel: Takluckehuven 40×40, 2-pack</t>
+          <t>AliExpress: US $47.29. Vår räkning: landad ca 684 kr, tänkt butikspris 1499 kr. Originaltitel: Värmepumpsskyddet i aluminium</t>
         </is>
       </c>
       <c r="H17" s="13" t="n"/>
@@ -1559,7 +1559,7 @@
       <c r="M17" s="14" t="n"/>
       <c r="N17" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012828233566.html</t>
+          <t>https://www.aliexpress.com/item/1005012880367856.html</t>
         </is>
       </c>
       <c r="Q17" s="18" t="n"/>
@@ -1709,12 +1709,12 @@
       <c r="A21" s="10" t="n"/>
       <c r="D21" s="18" t="inlineStr">
         <is>
-          <t>Gårdshundens plastkoja</t>
+          <t>Takluckehuven 40×40, 2-pack</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $32.77. Vår räkning: landad ca 474 kr, tänkt butikspris 999 kr. Originaltitel: Gårdshundens plastkoja</t>
+          <t>AliExpress: US $4.75. Vår räkning: landad ca 138 kr, tänkt butikspris 499 kr. Originaltitel: Takluckehuven 40×40, 2-pack</t>
         </is>
       </c>
       <c r="H21" s="13" t="n"/>
@@ -1729,7 +1729,7 @@
       <c r="M21" s="14" t="n"/>
       <c r="N21" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005010577271235.html</t>
+          <t>https://www.aliexpress.com/item/1005012828233566.html</t>
         </is>
       </c>
       <c r="Q21" s="18" t="n"/>
@@ -1879,12 +1879,12 @@
       <c r="A25" s="10" t="n"/>
       <c r="D25" s="18" t="inlineStr">
         <is>
-          <t>Isfria vattenskålen 2,2 L</t>
+          <t>Snöskyffeln för Makita-batteri</t>
         </is>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $27.09. Vår räkning: landad ca 392 kr, tänkt butikspris 699 kr. Originaltitel: Isfria vattenskålen 2,2 L</t>
+          <t>AliExpress: US $78.87. Vår räkning: landad ca 1140 kr, tänkt butikspris 1799 kr. Originaltitel: Snöskyffeln för Makita-batteri</t>
         </is>
       </c>
       <c r="H25" s="13" t="n"/>
@@ -1899,7 +1899,7 @@
       <c r="M25" s="14" t="n"/>
       <c r="N25" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012917988362.html</t>
+          <t>https://www.aliexpress.com/item/1005008160433396.html</t>
         </is>
       </c>
       <c r="Q25" s="18" t="n"/>
@@ -2049,12 +2049,12 @@
       <c r="A29" s="10" t="n"/>
       <c r="D29" s="18" t="inlineStr">
         <is>
-          <t>Viltsläden — rullbar dragmatta</t>
+          <t>Kajakhållaren för vägg, 2-pack</t>
         </is>
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $25.29. Vår räkning: landad ca 366 kr, tänkt butikspris 649 kr. Originaltitel: Viltsläden — rullbar dragmatta</t>
+          <t>AliExpress: US $15.95. Vår räkning: landad ca 231 kr, tänkt butikspris 499 kr. Originaltitel: Kajakhållaren för vägg, 2-pack</t>
         </is>
       </c>
       <c r="H29" s="13" t="n"/>
@@ -2069,7 +2069,7 @@
       <c r="M29" s="14" t="n"/>
       <c r="N29" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005008510065407.html</t>
+          <t>https://www.aliexpress.com/item/1005013089300340.html</t>
         </is>
       </c>
       <c r="Q29" s="18" t="n"/>
@@ -2219,12 +2219,12 @@
       <c r="A33" s="10" t="n"/>
       <c r="D33" s="18" t="inlineStr">
         <is>
-          <t>ATV-kapellet Heavy Duty</t>
+          <t>Värmesitsen för älgpasset</t>
         </is>
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $30.3. Vår räkning: landad ca 438 kr, tänkt butikspris 899 kr. Originaltitel: ATV-kapellet Heavy Duty</t>
+          <t>AliExpress: US $15.75. Vår räkning: landad ca 228 kr, tänkt butikspris 599 kr. Originaltitel: Värmesitsen för älgpasset</t>
         </is>
       </c>
       <c r="H33" s="13" t="n"/>
@@ -2239,7 +2239,7 @@
       <c r="M33" s="14" t="n"/>
       <c r="N33" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012520126605.html</t>
+          <t>https://www.aliexpress.com/item/1005007989005160.html</t>
         </is>
       </c>
       <c r="Q33" s="18" t="n"/>
@@ -2389,12 +2389,12 @@
       <c r="A37" s="10" t="n"/>
       <c r="D37" s="18" t="inlineStr">
         <is>
-          <t>Adventskalender Dinosaurier 24 figurer</t>
+          <t>Gårdshundens plastkoja</t>
         </is>
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $18.49. Vår räkning: landad ca 268 kr, tänkt butikspris 499 kr. Originaltitel: Adventskalender Dinosaurier 24 figurer</t>
+          <t>AliExpress: US $32.77. Vår räkning: landad ca 474 kr, tänkt butikspris 999 kr. Originaltitel: Gårdshundens plastkoja</t>
         </is>
       </c>
       <c r="H37" s="13" t="n"/>
@@ -2409,7 +2409,7 @@
       <c r="M37" s="14" t="n"/>
       <c r="N37" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005009776332625.html</t>
+          <t>https://www.aliexpress.com/item/1005010577271235.html</t>
         </is>
       </c>
       <c r="Q37" s="18" t="n"/>
@@ -2559,12 +2559,12 @@
       <c r="A41" s="10" t="n"/>
       <c r="D41" s="18" t="inlineStr">
         <is>
-          <t>Hjulskydden 4-pack husvagn/släp</t>
+          <t>Vedställsbeslaget 2-pack (egna reglar)</t>
         </is>
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $21.55. Vår räkning: landad ca 312 kr, tänkt butikspris 599 kr. Originaltitel: Hjulskydden 4-pack husvagn/släp</t>
+          <t>AliExpress: US $14.73. Vår räkning: landad ca 213 kr, tänkt butikspris 449 kr. Originaltitel: Vedställsbeslaget 2-pack (egna reglar)</t>
         </is>
       </c>
       <c r="H41" s="13" t="n"/>
@@ -2579,7 +2579,7 @@
       <c r="M41" s="14" t="n"/>
       <c r="N41" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005007500952009.html</t>
+          <t>https://www.aliexpress.com/item/1005008516015977.html</t>
         </is>
       </c>
       <c r="Q41" s="18" t="n"/>
@@ -2729,12 +2729,12 @@
       <c r="A45" s="10" t="n"/>
       <c r="D45" s="18" t="inlineStr">
         <is>
-          <t>Motorlåset rostfritt utombordare</t>
+          <t>Isfria vattenskålen 2,2 L</t>
         </is>
       </c>
       <c r="E45" s="12" t="inlineStr">
         <is>
-          <t>AliExpress: US $22.69. Vår räkning: landad ca 328 kr, tänkt butikspris 599 kr. Originaltitel: Motorlåset rostfritt utombordare</t>
+          <t>AliExpress: US $27.09. Vår räkning: landad ca 392 kr, tänkt butikspris 699 kr. Originaltitel: Isfria vattenskålen 2,2 L</t>
         </is>
       </c>
       <c r="H45" s="13" t="n"/>
@@ -2749,7 +2749,7 @@
       <c r="M45" s="14" t="n"/>
       <c r="N45" s="17" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/1005012502596910.html</t>
+          <t>https://www.aliexpress.com/item/1005012917988362.html</t>
         </is>
       </c>
       <c r="Q45" s="18" t="n"/>
@@ -2895,22 +2895,686 @@
       <c r="AT48" s="35" t="n"/>
       <c r="AU48" s="35" t="n"/>
     </row>
-    <row r="49" ht="15.75" customHeight="1" s="71"/>
-    <row r="50" ht="15.75" customHeight="1" s="71"/>
-    <row r="51" ht="15.75" customHeight="1" s="71"/>
-    <row r="52" ht="15.75" customHeight="1" s="71"/>
-    <row r="53" ht="15.75" customHeight="1" s="71"/>
-    <row r="54" ht="15.75" customHeight="1" s="71"/>
-    <row r="55" ht="15.75" customHeight="1" s="71"/>
-    <row r="56" ht="15.75" customHeight="1" s="71"/>
-    <row r="57" ht="15.75" customHeight="1" s="71"/>
-    <row r="58" ht="15.75" customHeight="1" s="71"/>
-    <row r="59" ht="15.75" customHeight="1" s="71"/>
-    <row r="60" ht="15.75" customHeight="1" s="71"/>
-    <row r="61" ht="15.75" customHeight="1" s="71"/>
-    <row r="62" ht="15.75" customHeight="1" s="71"/>
-    <row r="63" ht="15.75" customHeight="1" s="71"/>
-    <row r="64" ht="15.75" customHeight="1" s="71"/>
+    <row r="49" ht="24" customHeight="1" s="71">
+      <c r="A49" s="10" t="n"/>
+      <c r="D49" s="18" t="inlineStr">
+        <is>
+          <t>Fågelmataren med kamera (5MP, solcell)</t>
+        </is>
+      </c>
+      <c r="E49" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $77.19. Vår räkning: landad ca 1116 kr, tänkt butikspris 1499 kr. Originaltitel: Fågelmataren med kamera (5MP, solcell)</t>
+        </is>
+      </c>
+      <c r="H49" s="13" t="n"/>
+      <c r="I49" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J49" s="15" t="n"/>
+      <c r="K49" s="15" t="n"/>
+      <c r="L49" s="16" t="n"/>
+      <c r="M49" s="14" t="n"/>
+      <c r="N49" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005012746702398.html</t>
+        </is>
+      </c>
+      <c r="Q49" s="18" t="n"/>
+      <c r="R49" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S49" s="15" t="n"/>
+      <c r="T49" s="15" t="n"/>
+      <c r="U49" s="16" t="n"/>
+      <c r="V49" s="48" t="n"/>
+      <c r="W49" s="48" t="n"/>
+      <c r="X49" s="21" t="n"/>
+      <c r="Y49" s="15" t="n"/>
+      <c r="Z49" s="15" t="n"/>
+      <c r="AA49" s="16" t="n"/>
+      <c r="AB49" s="48" t="n"/>
+      <c r="AC49" s="48" t="n"/>
+      <c r="AD49" s="22" t="n"/>
+      <c r="AE49" s="15" t="n"/>
+      <c r="AF49" s="15" t="n"/>
+      <c r="AG49" s="16" t="n"/>
+      <c r="AH49" s="48" t="n"/>
+      <c r="AI49" s="48" t="n"/>
+      <c r="AJ49" s="23" t="n"/>
+      <c r="AK49" s="15" t="n"/>
+      <c r="AL49" s="15" t="n"/>
+      <c r="AM49" s="16" t="n"/>
+      <c r="AN49" s="25" t="n"/>
+      <c r="AO49" s="48" t="n"/>
+      <c r="AP49" s="23" t="n"/>
+      <c r="AQ49" s="15" t="n"/>
+      <c r="AR49" s="15" t="n"/>
+      <c r="AS49" s="16" t="n"/>
+      <c r="AT49" s="25" t="n"/>
+      <c r="AU49" s="26" t="n"/>
+    </row>
+    <row r="50" ht="25.5" customHeight="1" s="71">
+      <c r="D50" s="18" t="n"/>
+      <c r="J50" s="15" t="n"/>
+      <c r="K50" s="15" t="n"/>
+      <c r="L50" s="16" t="n"/>
+      <c r="R50" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S50" s="15" t="n"/>
+      <c r="T50" s="15" t="n"/>
+      <c r="U50" s="16" t="n"/>
+      <c r="X50" s="21" t="n"/>
+      <c r="Y50" s="15" t="n"/>
+      <c r="Z50" s="15" t="n"/>
+      <c r="AA50" s="16" t="n"/>
+      <c r="AD50" s="22" t="n"/>
+      <c r="AE50" s="15" t="n"/>
+      <c r="AF50" s="15" t="n"/>
+      <c r="AG50" s="16" t="n"/>
+      <c r="AH50" s="48" t="n"/>
+      <c r="AI50" s="48" t="n"/>
+      <c r="AJ50" s="23" t="n"/>
+      <c r="AK50" s="15" t="n"/>
+      <c r="AL50" s="15" t="n"/>
+      <c r="AM50" s="16" t="n"/>
+      <c r="AP50" s="23" t="n"/>
+      <c r="AQ50" s="15" t="n"/>
+      <c r="AR50" s="15" t="n"/>
+      <c r="AS50" s="16" t="n"/>
+    </row>
+    <row r="51" s="71">
+      <c r="D51" s="18" t="n"/>
+      <c r="J51" s="15" t="n"/>
+      <c r="K51" s="15" t="n"/>
+      <c r="L51" s="16" t="n"/>
+      <c r="R51" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S51" s="15" t="n"/>
+      <c r="T51" s="15" t="n"/>
+      <c r="U51" s="16" t="n"/>
+      <c r="X51" s="21" t="n"/>
+      <c r="Y51" s="15" t="n"/>
+      <c r="Z51" s="15" t="n"/>
+      <c r="AA51" s="16" t="n"/>
+      <c r="AD51" s="22" t="n"/>
+      <c r="AE51" s="15" t="n"/>
+      <c r="AF51" s="15" t="n"/>
+      <c r="AG51" s="16" t="n"/>
+      <c r="AH51" s="48" t="n"/>
+      <c r="AI51" s="48" t="n"/>
+      <c r="AJ51" s="23" t="n"/>
+      <c r="AK51" s="15" t="n"/>
+      <c r="AL51" s="15" t="n"/>
+      <c r="AM51" s="16" t="n"/>
+      <c r="AP51" s="23" t="n"/>
+      <c r="AQ51" s="15" t="n"/>
+      <c r="AR51" s="15" t="n"/>
+      <c r="AS51" s="16" t="n"/>
+    </row>
+    <row r="52" ht="6.75" customHeight="1" s="71">
+      <c r="A52" s="27" t="n"/>
+      <c r="B52" s="27" t="n"/>
+      <c r="C52" s="27" t="n"/>
+      <c r="D52" s="27" t="n"/>
+      <c r="E52" s="27" t="n"/>
+      <c r="F52" s="27" t="n"/>
+      <c r="G52" s="27" t="n"/>
+      <c r="H52" s="35" t="n"/>
+      <c r="I52" s="35" t="n"/>
+      <c r="J52" s="36" t="n"/>
+      <c r="K52" s="36" t="n"/>
+      <c r="L52" s="36" t="n"/>
+      <c r="M52" s="35" t="n"/>
+      <c r="N52" s="30" t="n"/>
+      <c r="O52" s="30" t="n"/>
+      <c r="P52" s="30" t="n"/>
+      <c r="Q52" s="30" t="n"/>
+      <c r="R52" s="35" t="n"/>
+      <c r="S52" s="35" t="n"/>
+      <c r="T52" s="35" t="n"/>
+      <c r="U52" s="35" t="n"/>
+      <c r="V52" s="35" t="n"/>
+      <c r="W52" s="35" t="n"/>
+      <c r="X52" s="31" t="n"/>
+      <c r="Y52" s="35" t="n"/>
+      <c r="Z52" s="35" t="n"/>
+      <c r="AA52" s="36" t="n"/>
+      <c r="AB52" s="35" t="n"/>
+      <c r="AC52" s="35" t="n"/>
+      <c r="AD52" s="32" t="n"/>
+      <c r="AE52" s="35" t="n"/>
+      <c r="AF52" s="35" t="n"/>
+      <c r="AG52" s="36" t="n"/>
+      <c r="AH52" s="35" t="n"/>
+      <c r="AI52" s="35" t="n"/>
+      <c r="AJ52" s="34" t="n"/>
+      <c r="AK52" s="35" t="n"/>
+      <c r="AL52" s="35" t="n"/>
+      <c r="AM52" s="36" t="n"/>
+      <c r="AN52" s="35" t="n"/>
+      <c r="AO52" s="35" t="n"/>
+      <c r="AP52" s="34" t="n"/>
+      <c r="AQ52" s="35" t="n"/>
+      <c r="AR52" s="35" t="n"/>
+      <c r="AS52" s="36" t="n"/>
+      <c r="AT52" s="35" t="n"/>
+      <c r="AU52" s="35" t="n"/>
+    </row>
+    <row r="53" ht="24" customHeight="1" s="71">
+      <c r="A53" s="10" t="n"/>
+      <c r="D53" s="18" t="inlineStr">
+        <is>
+          <t>ATV-kapellet Heavy Duty</t>
+        </is>
+      </c>
+      <c r="E53" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $30.3. Vår räkning: landad ca 438 kr, tänkt butikspris 899 kr. Originaltitel: ATV-kapellet Heavy Duty</t>
+        </is>
+      </c>
+      <c r="H53" s="13" t="n"/>
+      <c r="I53" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J53" s="15" t="n"/>
+      <c r="K53" s="15" t="n"/>
+      <c r="L53" s="16" t="n"/>
+      <c r="M53" s="14" t="n"/>
+      <c r="N53" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005012520126605.html</t>
+        </is>
+      </c>
+      <c r="Q53" s="18" t="n"/>
+      <c r="R53" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S53" s="15" t="n"/>
+      <c r="T53" s="15" t="n"/>
+      <c r="U53" s="16" t="n"/>
+      <c r="V53" s="48" t="n"/>
+      <c r="W53" s="48" t="n"/>
+      <c r="X53" s="21" t="n"/>
+      <c r="Y53" s="15" t="n"/>
+      <c r="Z53" s="15" t="n"/>
+      <c r="AA53" s="16" t="n"/>
+      <c r="AB53" s="48" t="n"/>
+      <c r="AC53" s="48" t="n"/>
+      <c r="AD53" s="22" t="n"/>
+      <c r="AE53" s="15" t="n"/>
+      <c r="AF53" s="15" t="n"/>
+      <c r="AG53" s="16" t="n"/>
+      <c r="AH53" s="48" t="n"/>
+      <c r="AI53" s="48" t="n"/>
+      <c r="AJ53" s="23" t="n"/>
+      <c r="AK53" s="15" t="n"/>
+      <c r="AL53" s="15" t="n"/>
+      <c r="AM53" s="16" t="n"/>
+      <c r="AN53" s="25" t="n"/>
+      <c r="AO53" s="48" t="n"/>
+      <c r="AP53" s="23" t="n"/>
+      <c r="AQ53" s="15" t="n"/>
+      <c r="AR53" s="15" t="n"/>
+      <c r="AS53" s="16" t="n"/>
+      <c r="AT53" s="25" t="n"/>
+      <c r="AU53" s="26" t="n"/>
+    </row>
+    <row r="54" ht="25.5" customHeight="1" s="71">
+      <c r="D54" s="18" t="n"/>
+      <c r="J54" s="15" t="n"/>
+      <c r="K54" s="15" t="n"/>
+      <c r="L54" s="16" t="n"/>
+      <c r="R54" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S54" s="15" t="n"/>
+      <c r="T54" s="15" t="n"/>
+      <c r="U54" s="16" t="n"/>
+      <c r="X54" s="21" t="n"/>
+      <c r="Y54" s="15" t="n"/>
+      <c r="Z54" s="15" t="n"/>
+      <c r="AA54" s="16" t="n"/>
+      <c r="AD54" s="22" t="n"/>
+      <c r="AE54" s="15" t="n"/>
+      <c r="AF54" s="15" t="n"/>
+      <c r="AG54" s="16" t="n"/>
+      <c r="AH54" s="48" t="n"/>
+      <c r="AI54" s="48" t="n"/>
+      <c r="AJ54" s="23" t="n"/>
+      <c r="AK54" s="15" t="n"/>
+      <c r="AL54" s="15" t="n"/>
+      <c r="AM54" s="16" t="n"/>
+      <c r="AP54" s="23" t="n"/>
+      <c r="AQ54" s="15" t="n"/>
+      <c r="AR54" s="15" t="n"/>
+      <c r="AS54" s="16" t="n"/>
+    </row>
+    <row r="55" s="71">
+      <c r="D55" s="18" t="n"/>
+      <c r="J55" s="15" t="n"/>
+      <c r="K55" s="15" t="n"/>
+      <c r="L55" s="16" t="n"/>
+      <c r="R55" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S55" s="15" t="n"/>
+      <c r="T55" s="15" t="n"/>
+      <c r="U55" s="16" t="n"/>
+      <c r="X55" s="21" t="n"/>
+      <c r="Y55" s="15" t="n"/>
+      <c r="Z55" s="15" t="n"/>
+      <c r="AA55" s="16" t="n"/>
+      <c r="AD55" s="22" t="n"/>
+      <c r="AE55" s="15" t="n"/>
+      <c r="AF55" s="15" t="n"/>
+      <c r="AG55" s="16" t="n"/>
+      <c r="AH55" s="48" t="n"/>
+      <c r="AI55" s="48" t="n"/>
+      <c r="AJ55" s="23" t="n"/>
+      <c r="AK55" s="15" t="n"/>
+      <c r="AL55" s="15" t="n"/>
+      <c r="AM55" s="16" t="n"/>
+      <c r="AP55" s="23" t="n"/>
+      <c r="AQ55" s="15" t="n"/>
+      <c r="AR55" s="15" t="n"/>
+      <c r="AS55" s="16" t="n"/>
+    </row>
+    <row r="56" ht="6.75" customHeight="1" s="71">
+      <c r="A56" s="27" t="n"/>
+      <c r="B56" s="27" t="n"/>
+      <c r="C56" s="27" t="n"/>
+      <c r="D56" s="27" t="n"/>
+      <c r="E56" s="27" t="n"/>
+      <c r="F56" s="27" t="n"/>
+      <c r="G56" s="27" t="n"/>
+      <c r="H56" s="35" t="n"/>
+      <c r="I56" s="35" t="n"/>
+      <c r="J56" s="36" t="n"/>
+      <c r="K56" s="36" t="n"/>
+      <c r="L56" s="36" t="n"/>
+      <c r="M56" s="35" t="n"/>
+      <c r="N56" s="30" t="n"/>
+      <c r="O56" s="30" t="n"/>
+      <c r="P56" s="30" t="n"/>
+      <c r="Q56" s="30" t="n"/>
+      <c r="R56" s="35" t="n"/>
+      <c r="S56" s="35" t="n"/>
+      <c r="T56" s="35" t="n"/>
+      <c r="U56" s="35" t="n"/>
+      <c r="V56" s="35" t="n"/>
+      <c r="W56" s="35" t="n"/>
+      <c r="X56" s="31" t="n"/>
+      <c r="Y56" s="35" t="n"/>
+      <c r="Z56" s="35" t="n"/>
+      <c r="AA56" s="36" t="n"/>
+      <c r="AB56" s="35" t="n"/>
+      <c r="AC56" s="35" t="n"/>
+      <c r="AD56" s="32" t="n"/>
+      <c r="AE56" s="35" t="n"/>
+      <c r="AF56" s="35" t="n"/>
+      <c r="AG56" s="36" t="n"/>
+      <c r="AH56" s="35" t="n"/>
+      <c r="AI56" s="35" t="n"/>
+      <c r="AJ56" s="34" t="n"/>
+      <c r="AK56" s="35" t="n"/>
+      <c r="AL56" s="35" t="n"/>
+      <c r="AM56" s="36" t="n"/>
+      <c r="AN56" s="35" t="n"/>
+      <c r="AO56" s="35" t="n"/>
+      <c r="AP56" s="34" t="n"/>
+      <c r="AQ56" s="35" t="n"/>
+      <c r="AR56" s="35" t="n"/>
+      <c r="AS56" s="36" t="n"/>
+      <c r="AT56" s="35" t="n"/>
+      <c r="AU56" s="35" t="n"/>
+    </row>
+    <row r="57" ht="24" customHeight="1" s="71">
+      <c r="A57" s="10" t="n"/>
+      <c r="D57" s="18" t="inlineStr">
+        <is>
+          <t>Täljsetet 30 delar i väska</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $38.81. Vår räkning: landad ca 561 kr, tänkt butikspris 899 kr. Originaltitel: Täljsetet 30 delar i väska</t>
+        </is>
+      </c>
+      <c r="H57" s="13" t="n"/>
+      <c r="I57" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J57" s="15" t="n"/>
+      <c r="K57" s="15" t="n"/>
+      <c r="L57" s="16" t="n"/>
+      <c r="M57" s="14" t="n"/>
+      <c r="N57" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005012818225884.html</t>
+        </is>
+      </c>
+      <c r="Q57" s="18" t="n"/>
+      <c r="R57" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S57" s="15" t="n"/>
+      <c r="T57" s="15" t="n"/>
+      <c r="U57" s="16" t="n"/>
+      <c r="V57" s="48" t="n"/>
+      <c r="W57" s="48" t="n"/>
+      <c r="X57" s="21" t="n"/>
+      <c r="Y57" s="15" t="n"/>
+      <c r="Z57" s="15" t="n"/>
+      <c r="AA57" s="16" t="n"/>
+      <c r="AB57" s="48" t="n"/>
+      <c r="AC57" s="48" t="n"/>
+      <c r="AD57" s="22" t="n"/>
+      <c r="AE57" s="15" t="n"/>
+      <c r="AF57" s="15" t="n"/>
+      <c r="AG57" s="16" t="n"/>
+      <c r="AH57" s="48" t="n"/>
+      <c r="AI57" s="48" t="n"/>
+      <c r="AJ57" s="23" t="n"/>
+      <c r="AK57" s="15" t="n"/>
+      <c r="AL57" s="15" t="n"/>
+      <c r="AM57" s="16" t="n"/>
+      <c r="AN57" s="25" t="n"/>
+      <c r="AO57" s="48" t="n"/>
+      <c r="AP57" s="23" t="n"/>
+      <c r="AQ57" s="15" t="n"/>
+      <c r="AR57" s="15" t="n"/>
+      <c r="AS57" s="16" t="n"/>
+      <c r="AT57" s="25" t="n"/>
+      <c r="AU57" s="26" t="n"/>
+    </row>
+    <row r="58" ht="25.5" customHeight="1" s="71">
+      <c r="D58" s="18" t="n"/>
+      <c r="J58" s="15" t="n"/>
+      <c r="K58" s="15" t="n"/>
+      <c r="L58" s="16" t="n"/>
+      <c r="R58" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S58" s="15" t="n"/>
+      <c r="T58" s="15" t="n"/>
+      <c r="U58" s="16" t="n"/>
+      <c r="X58" s="21" t="n"/>
+      <c r="Y58" s="15" t="n"/>
+      <c r="Z58" s="15" t="n"/>
+      <c r="AA58" s="16" t="n"/>
+      <c r="AD58" s="22" t="n"/>
+      <c r="AE58" s="15" t="n"/>
+      <c r="AF58" s="15" t="n"/>
+      <c r="AG58" s="16" t="n"/>
+      <c r="AH58" s="48" t="n"/>
+      <c r="AI58" s="48" t="n"/>
+      <c r="AJ58" s="23" t="n"/>
+      <c r="AK58" s="15" t="n"/>
+      <c r="AL58" s="15" t="n"/>
+      <c r="AM58" s="16" t="n"/>
+      <c r="AP58" s="23" t="n"/>
+      <c r="AQ58" s="15" t="n"/>
+      <c r="AR58" s="15" t="n"/>
+      <c r="AS58" s="16" t="n"/>
+    </row>
+    <row r="59" s="71">
+      <c r="D59" s="18" t="n"/>
+      <c r="J59" s="15" t="n"/>
+      <c r="K59" s="15" t="n"/>
+      <c r="L59" s="16" t="n"/>
+      <c r="R59" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S59" s="15" t="n"/>
+      <c r="T59" s="15" t="n"/>
+      <c r="U59" s="16" t="n"/>
+      <c r="X59" s="21" t="n"/>
+      <c r="Y59" s="15" t="n"/>
+      <c r="Z59" s="15" t="n"/>
+      <c r="AA59" s="16" t="n"/>
+      <c r="AD59" s="22" t="n"/>
+      <c r="AE59" s="15" t="n"/>
+      <c r="AF59" s="15" t="n"/>
+      <c r="AG59" s="16" t="n"/>
+      <c r="AH59" s="48" t="n"/>
+      <c r="AI59" s="48" t="n"/>
+      <c r="AJ59" s="23" t="n"/>
+      <c r="AK59" s="15" t="n"/>
+      <c r="AL59" s="15" t="n"/>
+      <c r="AM59" s="16" t="n"/>
+      <c r="AP59" s="23" t="n"/>
+      <c r="AQ59" s="15" t="n"/>
+      <c r="AR59" s="15" t="n"/>
+      <c r="AS59" s="16" t="n"/>
+    </row>
+    <row r="60" ht="6.75" customHeight="1" s="71">
+      <c r="A60" s="27" t="n"/>
+      <c r="B60" s="27" t="n"/>
+      <c r="C60" s="27" t="n"/>
+      <c r="D60" s="27" t="n"/>
+      <c r="E60" s="27" t="n"/>
+      <c r="F60" s="27" t="n"/>
+      <c r="G60" s="27" t="n"/>
+      <c r="H60" s="35" t="n"/>
+      <c r="I60" s="35" t="n"/>
+      <c r="J60" s="36" t="n"/>
+      <c r="K60" s="36" t="n"/>
+      <c r="L60" s="36" t="n"/>
+      <c r="M60" s="35" t="n"/>
+      <c r="N60" s="30" t="n"/>
+      <c r="O60" s="30" t="n"/>
+      <c r="P60" s="30" t="n"/>
+      <c r="Q60" s="30" t="n"/>
+      <c r="R60" s="35" t="n"/>
+      <c r="S60" s="35" t="n"/>
+      <c r="T60" s="35" t="n"/>
+      <c r="U60" s="35" t="n"/>
+      <c r="V60" s="35" t="n"/>
+      <c r="W60" s="35" t="n"/>
+      <c r="X60" s="31" t="n"/>
+      <c r="Y60" s="35" t="n"/>
+      <c r="Z60" s="35" t="n"/>
+      <c r="AA60" s="36" t="n"/>
+      <c r="AB60" s="35" t="n"/>
+      <c r="AC60" s="35" t="n"/>
+      <c r="AD60" s="32" t="n"/>
+      <c r="AE60" s="35" t="n"/>
+      <c r="AF60" s="35" t="n"/>
+      <c r="AG60" s="36" t="n"/>
+      <c r="AH60" s="35" t="n"/>
+      <c r="AI60" s="35" t="n"/>
+      <c r="AJ60" s="34" t="n"/>
+      <c r="AK60" s="35" t="n"/>
+      <c r="AL60" s="35" t="n"/>
+      <c r="AM60" s="36" t="n"/>
+      <c r="AN60" s="35" t="n"/>
+      <c r="AO60" s="35" t="n"/>
+      <c r="AP60" s="34" t="n"/>
+      <c r="AQ60" s="35" t="n"/>
+      <c r="AR60" s="35" t="n"/>
+      <c r="AS60" s="36" t="n"/>
+      <c r="AT60" s="35" t="n"/>
+      <c r="AU60" s="35" t="n"/>
+    </row>
+    <row r="61" ht="24" customHeight="1" s="71">
+      <c r="A61" s="10" t="n"/>
+      <c r="D61" s="18" t="inlineStr">
+        <is>
+          <t>Hjulskydden 4-pack husvagn/släp</t>
+        </is>
+      </c>
+      <c r="E61" s="12" t="inlineStr">
+        <is>
+          <t>AliExpress: US $21.55. Vår räkning: landad ca 312 kr, tänkt butikspris 599 kr. Originaltitel: Hjulskydden 4-pack husvagn/släp</t>
+        </is>
+      </c>
+      <c r="H61" s="13" t="n"/>
+      <c r="I61" s="14" t="inlineStr">
+        <is>
+          <t>SWEDEN</t>
+        </is>
+      </c>
+      <c r="J61" s="15" t="n"/>
+      <c r="K61" s="15" t="n"/>
+      <c r="L61" s="16" t="n"/>
+      <c r="M61" s="14" t="n"/>
+      <c r="N61" s="17" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.com/item/1005007500952009.html</t>
+        </is>
+      </c>
+      <c r="Q61" s="18" t="n"/>
+      <c r="R61" s="19" t="n">
+        <v>100</v>
+      </c>
+      <c r="S61" s="15" t="n"/>
+      <c r="T61" s="15" t="n"/>
+      <c r="U61" s="16" t="n"/>
+      <c r="V61" s="48" t="n"/>
+      <c r="W61" s="48" t="n"/>
+      <c r="X61" s="21" t="n"/>
+      <c r="Y61" s="15" t="n"/>
+      <c r="Z61" s="15" t="n"/>
+      <c r="AA61" s="16" t="n"/>
+      <c r="AB61" s="48" t="n"/>
+      <c r="AC61" s="48" t="n"/>
+      <c r="AD61" s="22" t="n"/>
+      <c r="AE61" s="15" t="n"/>
+      <c r="AF61" s="15" t="n"/>
+      <c r="AG61" s="16" t="n"/>
+      <c r="AH61" s="48" t="n"/>
+      <c r="AI61" s="48" t="n"/>
+      <c r="AJ61" s="23" t="n"/>
+      <c r="AK61" s="15" t="n"/>
+      <c r="AL61" s="15" t="n"/>
+      <c r="AM61" s="16" t="n"/>
+      <c r="AN61" s="25" t="n"/>
+      <c r="AO61" s="48" t="n"/>
+      <c r="AP61" s="23" t="n"/>
+      <c r="AQ61" s="15" t="n"/>
+      <c r="AR61" s="15" t="n"/>
+      <c r="AS61" s="16" t="n"/>
+      <c r="AT61" s="25" t="n"/>
+      <c r="AU61" s="26" t="n"/>
+    </row>
+    <row r="62" ht="25.5" customHeight="1" s="71">
+      <c r="D62" s="18" t="n"/>
+      <c r="J62" s="15" t="n"/>
+      <c r="K62" s="15" t="n"/>
+      <c r="L62" s="16" t="n"/>
+      <c r="R62" s="19" t="n">
+        <v>200</v>
+      </c>
+      <c r="S62" s="15" t="n"/>
+      <c r="T62" s="15" t="n"/>
+      <c r="U62" s="16" t="n"/>
+      <c r="X62" s="21" t="n"/>
+      <c r="Y62" s="15" t="n"/>
+      <c r="Z62" s="15" t="n"/>
+      <c r="AA62" s="16" t="n"/>
+      <c r="AD62" s="22" t="n"/>
+      <c r="AE62" s="15" t="n"/>
+      <c r="AF62" s="15" t="n"/>
+      <c r="AG62" s="16" t="n"/>
+      <c r="AH62" s="48" t="n"/>
+      <c r="AI62" s="48" t="n"/>
+      <c r="AJ62" s="23" t="n"/>
+      <c r="AK62" s="15" t="n"/>
+      <c r="AL62" s="15" t="n"/>
+      <c r="AM62" s="16" t="n"/>
+      <c r="AP62" s="23" t="n"/>
+      <c r="AQ62" s="15" t="n"/>
+      <c r="AR62" s="15" t="n"/>
+      <c r="AS62" s="16" t="n"/>
+    </row>
+    <row r="63" s="71">
+      <c r="D63" s="18" t="n"/>
+      <c r="J63" s="15" t="n"/>
+      <c r="K63" s="15" t="n"/>
+      <c r="L63" s="16" t="n"/>
+      <c r="R63" s="19" t="n">
+        <v>300</v>
+      </c>
+      <c r="S63" s="15" t="n"/>
+      <c r="T63" s="15" t="n"/>
+      <c r="U63" s="16" t="n"/>
+      <c r="X63" s="21" t="n"/>
+      <c r="Y63" s="15" t="n"/>
+      <c r="Z63" s="15" t="n"/>
+      <c r="AA63" s="16" t="n"/>
+      <c r="AD63" s="22" t="n"/>
+      <c r="AE63" s="15" t="n"/>
+      <c r="AF63" s="15" t="n"/>
+      <c r="AG63" s="16" t="n"/>
+      <c r="AH63" s="48" t="n"/>
+      <c r="AI63" s="48" t="n"/>
+      <c r="AJ63" s="23" t="n"/>
+      <c r="AK63" s="15" t="n"/>
+      <c r="AL63" s="15" t="n"/>
+      <c r="AM63" s="16" t="n"/>
+      <c r="AP63" s="23" t="n"/>
+      <c r="AQ63" s="15" t="n"/>
+      <c r="AR63" s="15" t="n"/>
+      <c r="AS63" s="16" t="n"/>
+    </row>
+    <row r="64" ht="6.75" customHeight="1" s="71">
+      <c r="A64" s="27" t="n"/>
+      <c r="B64" s="27" t="n"/>
+      <c r="C64" s="27" t="n"/>
+      <c r="D64" s="27" t="n"/>
+      <c r="E64" s="27" t="n"/>
+      <c r="F64" s="27" t="n"/>
+      <c r="G64" s="27" t="n"/>
+      <c r="H64" s="35" t="n"/>
+      <c r="I64" s="35" t="n"/>
+      <c r="J64" s="36" t="n"/>
+      <c r="K64" s="36" t="n"/>
+      <c r="L64" s="36" t="n"/>
+      <c r="M64" s="35" t="n"/>
+      <c r="N64" s="30" t="n"/>
+      <c r="O64" s="30" t="n"/>
+      <c r="P64" s="30" t="n"/>
+      <c r="Q64" s="30" t="n"/>
+      <c r="R64" s="35" t="n"/>
+      <c r="S64" s="35" t="n"/>
+      <c r="T64" s="35" t="n"/>
+      <c r="U64" s="35" t="n"/>
+      <c r="V64" s="35" t="n"/>
+      <c r="W64" s="35" t="n"/>
+      <c r="X64" s="31" t="n"/>
+      <c r="Y64" s="35" t="n"/>
+      <c r="Z64" s="35" t="n"/>
+      <c r="AA64" s="36" t="n"/>
+      <c r="AB64" s="35" t="n"/>
+      <c r="AC64" s="35" t="n"/>
+      <c r="AD64" s="32" t="n"/>
+      <c r="AE64" s="35" t="n"/>
+      <c r="AF64" s="35" t="n"/>
+      <c r="AG64" s="36" t="n"/>
+      <c r="AH64" s="35" t="n"/>
+      <c r="AI64" s="35" t="n"/>
+      <c r="AJ64" s="34" t="n"/>
+      <c r="AK64" s="35" t="n"/>
+      <c r="AL64" s="35" t="n"/>
+      <c r="AM64" s="36" t="n"/>
+      <c r="AN64" s="35" t="n"/>
+      <c r="AO64" s="35" t="n"/>
+      <c r="AP64" s="34" t="n"/>
+      <c r="AQ64" s="35" t="n"/>
+      <c r="AR64" s="35" t="n"/>
+      <c r="AS64" s="36" t="n"/>
+      <c r="AT64" s="35" t="n"/>
+      <c r="AU64" s="35" t="n"/>
+    </row>
     <row r="65" ht="15.75" customHeight="1" s="71"/>
     <row r="66" ht="15.75" customHeight="1" s="71"/>
     <row r="67" ht="15.75" customHeight="1" s="71"/>
@@ -3848,18 +4512,23 @@
     <row r="999" ht="15.75" customHeight="1" s="71"/>
     <row r="1000" ht="15.75" customHeight="1" s="71"/>
   </sheetData>
-  <mergeCells count="94">
+  <mergeCells count="122">
     <mergeCell ref="E5:G7"/>
     <mergeCell ref="H17:H19"/>
     <mergeCell ref="M21:M23"/>
     <mergeCell ref="L3:L4"/>
+    <mergeCell ref="M57:M59"/>
     <mergeCell ref="N5:P7"/>
     <mergeCell ref="M41:M43"/>
     <mergeCell ref="N33:P35"/>
     <mergeCell ref="A37:C39"/>
+    <mergeCell ref="Q57:Q59"/>
     <mergeCell ref="R3:W3"/>
     <mergeCell ref="A21:C23"/>
+    <mergeCell ref="I49:I51"/>
+    <mergeCell ref="N57:P59"/>
     <mergeCell ref="I3:I4"/>
+    <mergeCell ref="A57:C59"/>
     <mergeCell ref="Q41:Q43"/>
     <mergeCell ref="H5:H7"/>
     <mergeCell ref="A29:C31"/>
@@ -3871,14 +4540,19 @@
     <mergeCell ref="E25:G27"/>
     <mergeCell ref="AP3:AU3"/>
     <mergeCell ref="H21:H23"/>
+    <mergeCell ref="I53:I55"/>
     <mergeCell ref="M25:M27"/>
     <mergeCell ref="Q3:Q4"/>
+    <mergeCell ref="M61:M63"/>
     <mergeCell ref="E17:G19"/>
     <mergeCell ref="I37:I39"/>
+    <mergeCell ref="H57:H59"/>
     <mergeCell ref="Q9:Q11"/>
     <mergeCell ref="M45:M47"/>
     <mergeCell ref="I29:I31"/>
     <mergeCell ref="I13:I15"/>
+    <mergeCell ref="E61:G63"/>
+    <mergeCell ref="Q61:Q63"/>
     <mergeCell ref="M29:M31"/>
     <mergeCell ref="A1:AO1"/>
     <mergeCell ref="H33:H35"/>
@@ -3887,6 +4561,7 @@
     <mergeCell ref="A5:C7"/>
     <mergeCell ref="N3:P4"/>
     <mergeCell ref="H25:H27"/>
+    <mergeCell ref="I57:I59"/>
     <mergeCell ref="N9:P11"/>
     <mergeCell ref="I41:I43"/>
     <mergeCell ref="E21:G23"/>
@@ -3894,14 +4569,19 @@
     <mergeCell ref="K3:K4"/>
     <mergeCell ref="N45:P47"/>
     <mergeCell ref="I25:I27"/>
+    <mergeCell ref="A49:C51"/>
+    <mergeCell ref="N53:P55"/>
     <mergeCell ref="I33:I35"/>
+    <mergeCell ref="H61:H63"/>
     <mergeCell ref="I5:I7"/>
     <mergeCell ref="I17:I19"/>
     <mergeCell ref="A41:C43"/>
     <mergeCell ref="N37:P39"/>
     <mergeCell ref="X3:AC3"/>
     <mergeCell ref="M33:M35"/>
+    <mergeCell ref="E49:G51"/>
     <mergeCell ref="N21:P23"/>
+    <mergeCell ref="N61:P63"/>
     <mergeCell ref="H13:H15"/>
     <mergeCell ref="E3:G4"/>
     <mergeCell ref="A25:C27"/>
@@ -3913,27 +4593,39 @@
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="Q13:Q15"/>
     <mergeCell ref="N13:P15"/>
+    <mergeCell ref="I61:I63"/>
     <mergeCell ref="A17:C19"/>
     <mergeCell ref="M9:M11"/>
     <mergeCell ref="Q37:Q39"/>
+    <mergeCell ref="H53:H55"/>
     <mergeCell ref="Q21:Q23"/>
+    <mergeCell ref="N49:P51"/>
     <mergeCell ref="H3:H4"/>
+    <mergeCell ref="E53:G55"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="H9:H11"/>
     <mergeCell ref="E37:G39"/>
     <mergeCell ref="N41:P43"/>
     <mergeCell ref="A45:C47"/>
+    <mergeCell ref="H49:H51"/>
     <mergeCell ref="N25:P27"/>
     <mergeCell ref="M13:M15"/>
     <mergeCell ref="E29:G31"/>
+    <mergeCell ref="Q49:Q51"/>
+    <mergeCell ref="A61:C63"/>
     <mergeCell ref="E13:G15"/>
     <mergeCell ref="H37:H39"/>
+    <mergeCell ref="M53:M55"/>
     <mergeCell ref="Q25:Q27"/>
+    <mergeCell ref="E57:G59"/>
     <mergeCell ref="N29:P31"/>
     <mergeCell ref="I9:I11"/>
     <mergeCell ref="A33:C35"/>
+    <mergeCell ref="Q53:Q55"/>
     <mergeCell ref="E41:G43"/>
     <mergeCell ref="I45:I47"/>
+    <mergeCell ref="A53:C55"/>
+    <mergeCell ref="M49:M51"/>
     <mergeCell ref="A3:C4"/>
     <mergeCell ref="H41:H43"/>
     <mergeCell ref="Q5:Q7"/>

</xml_diff>